<commit_message>
fix: translate the files
</commit_message>
<xml_diff>
--- a/test-cases/test-summary.xlsx
+++ b/test-cases/test-summary.xlsx
@@ -443,7 +443,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HW06 API Testing — Test Summary</t>
+          <t>HW06 API Testing - Tổng hợp test case</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Suite chạy xanh — assertion của case known-bug kiểm hành vi quan sát (được gắn nhãn [BUG-*]); lỗi được đếm riêng ở cột Bugs.</t>
+          <t>Suite chạy xanh — assertion của case bug đã biết kiểm hành vi quan sát (được gắn nhãn [BUG-*]); lỗi được đếm riêng ở cột Bug.</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>AI-generated</t>
+          <t>AI sinh</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -518,22 +518,22 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Newman assertions</t>
+          <t>Số assertion Newman</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Không đạt</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Bugs</t>
+          <t>Bug</t>
         </is>
       </c>
     </row>
@@ -547,10 +547,10 @@
         <v>40</v>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E8" t="n">
         <v>45</v>
@@ -624,17 +624,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>Tổng</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
         <v>115</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>233</v>

</xml_diff>